<commit_message>
docs(uat): Hata Kaydi durumlari duzeltme turuna gore guncellendi
HATA-01..10: 8 kayit 'Cozuldu (deploy bekliyor)', HATA-06 alan
kaldirilarak kapandi, HATA-08 kod-dogru olarak kapandi. Developer
Note'lara fix ozetleri islendi.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat/IMGA-UAT.xlsx
+++ b/docs/uat/IMGA-UAT.xlsx
@@ -3810,12 +3810,12 @@
       </c>
       <c r="L3" s="40" t="inlineStr">
         <is>
-          <t>tenant_batch.py:447 log.exception(extra={'filename': ...}) — 'filename' rezerve LogRecord alanı → KeyError; BadZipFile FileParseError'a map'lenmeli. Repo genelinde extra={'filename'} taranmalı.</t>
+          <t>tenant_batch.py:447 log.exception(extra={'filename': ...}) — 'filename' rezerve LogRecord alanı → KeyError; BadZipFile FileParseError'a map'lenmeli. Repo genelinde extra={'filename'} taranmalı. | FIX 10.07: extra 'upload_filename' + file_parser._load_xlsx (BadZipFile/InvalidFileException → FileParseError, 400/parse_failed).</t>
         </is>
       </c>
       <c r="M3" s="39" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Çözüldü (deploy bekliyor)</t>
         </is>
       </c>
     </row>
@@ -3877,12 +3877,12 @@
       </c>
       <c r="L4" s="42" t="inlineStr">
         <is>
-          <t>imga-core override katmanı 'kargo' kelime eşleşmesiyle skoru eziyor; BERT skoru pozitifken tetiklenmemeli. Toplu yüklemede de aynı desen ('teşekkürler harika hizmet' → Olumsuz).</t>
+          <t>imga-core override katmanı 'kargo' kelime eşleşmesiyle skoru eziyor; BERT skoru pozitifken tetiklenmemeli. Toplu yüklemede de aynı desen ('teşekkürler harika hizmet' → Olumsuz). | FIX 10.07: TIER2_FALLBACK_STRONG_POSITIVE_SKIP=0.6 — BERT skoru ≥0.6 iken tier2 ateşlemez; testler + snapshot fikstürü eklendi.</t>
         </is>
       </c>
       <c r="M4" s="41" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Çözüldü (deploy bekliyor)</t>
         </is>
       </c>
     </row>
@@ -3944,12 +3944,12 @@
       </c>
       <c r="L5" s="40" t="inlineStr">
         <is>
-          <t>promote_to_ticket → _resolve_category_id('belirsiz') CategoryNotConfiguredError; belirsiz için fallback kategori gerekli. FE 409 detail'ini yansıtmalı.</t>
+          <t>promote_to_ticket → _resolve_category_id('belirsiz') CategoryNotConfiguredError; belirsiz için fallback kategori gerekli. FE 409 detail'ini yansıtmalı. | FIX 10.07: migration 0036 global 'belirsiz' kategorisi (promote artık 201); FE 409 mesajı API detail'ine göre ayrışıyor.</t>
         </is>
       </c>
       <c r="M5" s="39" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Çözüldü (deploy bekliyor)</t>
         </is>
       </c>
     </row>
@@ -4011,12 +4011,12 @@
       </c>
       <c r="L6" s="42" t="inlineStr">
         <is>
-          <t>Multipart preview/upload fetch'i apiRequest'in 401→refresh→retry sarmalayıcısına bağlanmalı.</t>
+          <t>Multipart preview/upload fetch'i apiRequest'in 401→refresh→retry sarmalayıcısına bağlanmalı. | FIX 10.07: preview apiRequest'e taşındı (FormData + 401→refresh→replay); blob indirmeler apiRawFetch ile aynı akışta.</t>
         </is>
       </c>
       <c r="M6" s="41" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Çözüldü (deploy bekliyor)</t>
         </is>
       </c>
     </row>
@@ -4078,12 +4078,12 @@
       </c>
       <c r="L7" s="40" t="inlineStr">
         <is>
-          <t>settings/users/page.tsx:158 '/invitations/' → '/invite/' olmalı. Karşılaştırma: tenant-create-dialog.tsx:366 doğru üretiyor. ANL-09 koşumunda canlıda doğrulandı.</t>
+          <t>settings/users/page.tsx:158 '/invitations/' → '/invite/' olmalı. Karşılaştırma: tenant-create-dialog.tsx:366 doğru üretiyor. ANL-09 koşumunda canlıda doğrulandı. | FIX 10.07: settings/users davet linki /invite/&lt;token&gt; üretir.</t>
         </is>
       </c>
       <c r="M7" s="39" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Çözüldü (deploy bekliyor)</t>
         </is>
       </c>
     </row>
@@ -4145,12 +4145,12 @@
       </c>
       <c r="L8" s="42" t="inlineStr">
         <is>
-          <t>Preview'un text tespiti 'Metin sütunu' input'uyla senkronlanmalı.</t>
+          <t>Preview'un text tespiti 'Metin sütunu' input'uyla senkronlanmalı. | 10.07: 'Metin sütunu' alanı üründen kaldırıldı; kolon artık backend'de otomatik çözülüyor (yorum → text fallback).</t>
         </is>
       </c>
       <c r="M8" s="41" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Kapandı (alan kaldırıldı)</t>
         </is>
       </c>
     </row>
@@ -4212,12 +4212,12 @@
       </c>
       <c r="L9" s="40" t="inlineStr">
         <is>
-          <t>Özel doğrulama mesajı eklenebilir (davranış doğru, metin kozmetik).</t>
+          <t>Özel doğrulama mesajı eklenebilir (davranış doğru, metin kozmetik). | FIX 10.07: form noValidate — mevcut Türkçe toast ('NPS 0 ile 10 arasında olmalı.') devrede.</t>
         </is>
       </c>
       <c r="M9" s="39" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Çözüldü (deploy bekliyor)</t>
         </is>
       </c>
     </row>
@@ -4279,12 +4279,12 @@
       </c>
       <c r="L10" s="42" t="inlineStr">
         <is>
-          <t>Content-Disposition başlığı / indirme adlandırması kontrol edilmeli.</t>
+          <t>Content-Disposition başlığı / indirme adlandırması kontrol edilmeli. | 10.07 incelemesi: BE Content-Disposition + FE a.download zaten doğru adı veriyor; gözlenen .tmp adlandırması test otomasyonu tarayıcı ortamı artefaktı.</t>
         </is>
       </c>
       <c r="M10" s="41" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Kapandı (kod doğru)</t>
         </is>
       </c>
     </row>
@@ -4346,12 +4346,12 @@
       </c>
       <c r="L11" s="40" t="inlineStr">
         <is>
-          <t>Durum → renk eşlemesi gözden geçirilmeli.</t>
+          <t>Durum → renk eşlemesi gözden geçirilmeli. | FIX 10.07: durum→renk eşlemesi (tamamlandı=yeşil, işleniyor=amber, başarısız=kırmızı, iptal=gri).</t>
         </is>
       </c>
       <c r="M11" s="39" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Çözüldü (deploy bekliyor)</t>
         </is>
       </c>
     </row>
@@ -4413,12 +4413,12 @@
       </c>
       <c r="L12" s="42" t="inlineStr">
         <is>
-          <t>ForbiddenNotice metni bağlama göre parametreleşebilir.</t>
+          <t>ForbiddenNotice metni bağlama göre parametreleşebilir. | FIX 10.07: ForbiddenNotice descKey prop'u; RequireRole level'a göre metin (write/admin/super).</t>
         </is>
       </c>
       <c r="M12" s="41" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Çözüldü (deploy bekliyor)</t>
         </is>
       </c>
     </row>

</xml_diff>